<commit_message>
After Party : corrections lineups Mer/Jeu/Ven/Sam
- Mercredi Playa : DREAMS -> PHILIPPE + ROH
- Jeudi Playa : ROH -> FABULOUS (DREAMS + FABULOUS)
- Vendredi Playa : + DJ ROH ; Kizomba PP : Jean-Emile -> Alex Salsarito
- Samedi Playa : + DJ PHILIPPE ; Kizomba PP : + DJ BLANQUILLO

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning_DJs_SBL2026.xlsx
+++ b/Planning_DJs_SBL2026.xlsx
@@ -1086,7 +1086,7 @@
       <c r="D9" s="14" t="inlineStr"/>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>DREAMS + ROH</t>
+          <t>PHILIPPE + ROH</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
@@ -1244,7 +1244,7 @@
       <c r="D17" s="14" t="inlineStr"/>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>DREAMS + ROH</t>
+          <t>DREAMS + FABULOUS</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
@@ -1400,12 +1400,12 @@
       <c r="D25" s="14" t="inlineStr"/>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>DREAMS + FABULOUS</t>
+          <t>DREAMS + FABULOUS + ROH</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>TREW + Jean-Emile</t>
+          <t>TREW + Alex Salsarito</t>
         </is>
       </c>
     </row>
@@ -1557,12 +1557,12 @@
       <c r="D33" s="14" t="inlineStr"/>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>DREAMS + FABULOUS</t>
+          <t>DREAMS + FABULOUS + PHILIPPE</t>
         </is>
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>TREW + Mikado San</t>
+          <t>TREW + Mikado San + BLANQUILLO</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C9" s="35" t="inlineStr">
         <is>
-          <t>DJ DREAMS + DJ ROH
+          <t>DJ PHILIPPE + DJ ROH
 (After — Playa)</t>
         </is>
       </c>
@@ -1803,7 +1803,7 @@
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ℹ️  After Party Playa : DJ DREAMS + DJ ROH
+          <t xml:space="preserve">  ℹ️  After Party Playa : DJ PHILIPPE + DJ ROH
 After Party Kizomba (Park Place) : DJ TREW + DJ FABULOUS</t>
         </is>
       </c>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="C12" s="35" t="inlineStr">
         <is>
-          <t>DJ DREAMS + DJ ROH
+          <t>DJ DREAMS + DJ FABULOUS
 (After — Playa)</t>
         </is>
       </c>
@@ -2027,7 +2027,7 @@
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ℹ️  After Party Playa : DJ DREAMS + DJ ROH
+          <t xml:space="preserve">  ℹ️  After Party Playa : DJ DREAMS + DJ FABULOUS
 After Party Kizomba (Park Place) : DJ FABULOUS + DJ TREW</t>
         </is>
       </c>
@@ -2231,13 +2231,13 @@
       </c>
       <c r="C11" s="35" t="inlineStr">
         <is>
-          <t>DJ DREAMS + DJ FABULOUS
+          <t>DJ DREAMS + DJ FABULOUS + DJ ROH
 (After — Playa)</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
         <is>
-          <t>DJ TREW + DJ Jean-Emile
+          <t>DJ TREW + DJ Alex Salsarito
 (After Kizomba — Park Place)</t>
         </is>
       </c>
@@ -2245,8 +2245,8 @@
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ℹ️  After Party Playa : DJ DREAMS + DJ FABULOUS
-After Party Kizomba (Park Place) : DJ TREW + DJ Jean-Emile</t>
+          <t xml:space="preserve">  ℹ️  After Party Playa : DJ DREAMS + DJ FABULOUS + DJ ROH
+After Party Kizomba (Park Place) : DJ TREW + DJ Alex Salsarito</t>
         </is>
       </c>
     </row>
@@ -2455,13 +2455,13 @@
       </c>
       <c r="C12" s="35" t="inlineStr">
         <is>
-          <t>DJ DREAMS + DJ FABULOUS
+          <t>DJ DREAMS + DJ FABULOUS + DJ PHILIPPE
 (After — Playa)</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
         <is>
-          <t>DJ TREW + DJ Mikado San
+          <t>DJ TREW + DJ Mikado San + DJ BLANQUILLO
 (After Kizomba — Park Place)</t>
         </is>
       </c>
@@ -2469,8 +2469,8 @@
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ℹ️  After Party Playa : DJ DREAMS + DJ FABULOUS
-After Party Kizomba (Park Place) : DJ TREW + DJ Mikado San
+          <t xml:space="preserve">  ℹ️  After Party Playa : DJ DREAMS + DJ FABULOUS + DJ PHILIPPE
+After Party Kizomba (Park Place) : DJ TREW + DJ Mikado San + DJ BLANQUILLO
 ⚠️ Heure de fin à définir (au-delà de 04h autorisé)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Jeudi After Kizomba : FABULOUS -> Mikado San + TREW
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planning_DJs_SBL2026.xlsx
+++ b/Planning_DJs_SBL2026.xlsx
@@ -1249,7 +1249,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>FABULOUS + TREW</t>
+          <t>Mikado San + TREW</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="D12" s="36" t="inlineStr">
         <is>
-          <t>DJ FABULOUS + DJ TREW
+          <t>DJ Mikado San + DJ TREW
 (After Kizomba — Park Place)</t>
         </is>
       </c>
@@ -2028,7 +2028,7 @@
       <c r="A14" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  ℹ️  After Party Playa : DJ DREAMS + DJ FABULOUS
-After Party Kizomba (Park Place) : DJ FABULOUS + DJ TREW</t>
+After Party Kizomba (Park Place) : DJ Mikado San + DJ TREW</t>
         </is>
       </c>
     </row>

</xml_diff>